<commit_message>
Fix knowledge summary popover interaction
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R718d9dd079624920"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R856f747d89b44109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R6282a6aa09d045fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R6dced67a818d4dae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="Rc8ec823ccec442bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="Rd953edf9f8f34e96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Rce79e66bf62a434d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R0b8fcd57d70d4cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="Rdd5f0e6d19934c66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="Re394116a46484fcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Rbe75ccd134834960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R68de500256044901"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="Rc1992003f3aa4c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R101b17cfe78641e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R36aab189cd394c6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R0c4542f8f7ec4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="Rce87ebf8b7464509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Rc75e6b01fefe45ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="Rd37b1a7de5124cf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R7047ec25bc4d4120"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R55ae647cbfe445ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="R9e91cd9519dc4923"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Render markdown in knowledge summary popovers
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R68de500256044901"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="Rc1992003f3aa4c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R101b17cfe78641e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R36aab189cd394c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R0c4542f8f7ec4669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="Rce87ebf8b7464509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Rc75e6b01fefe45ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="Rd37b1a7de5124cf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R7047ec25bc4d4120"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R55ae647cbfe445ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="R9e91cd9519dc4923"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R037f1b83e8184481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R913b27447d05408c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Recb0522090e44c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R5d30e3caa25f45fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R62a6a99174b24a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="Re5f0f7e71cc64365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="R44e127989089455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="Rfe5cac1becfb4c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R5d409feb1f0f4806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R68b44e31f2204883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Raef4d14a8184488c"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add policy markdown extraction and knowledge browser
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R037f1b83e8184481"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R913b27447d05408c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Recb0522090e44c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R5d30e3caa25f45fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R62a6a99174b24a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="Re5f0f7e71cc64365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="R44e127989089455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="Rfe5cac1becfb4c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R5d409feb1f0f4806"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R68b44e31f2204883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Raef4d14a8184488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="Rb7ad366e8da14009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R05420c45ad5d4019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R32a7b5ffb9e546d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R23a774dffdee45c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R345af8af361c42cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R210201cc28d34b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Rf1bcfa65341f4375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R350139e745064551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R77bf6428b42545e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="Ra544721900914e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Rd5d0f29e89814227"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -965,6 +965,20 @@
         <x:v>优化网页头部、搜索和页签布局，删除当前页描述区域，增加导出 Excel 按钮，并固化所有知识新增、更新必须写入更新记录的维护规则。</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>更新</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>policyDocuments</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>新增政策正文及附件 Markdown 提取能力，固化 OCRmyPDF + Tesseract 本地 OCR 方案，已为当前 14 个政策文件及 5 个附件生成 Markdown 原文，并为网页新增知识浏览入口。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Force OCR for sparse scanned policy PDFs
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="Rb7ad366e8da14009"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R05420c45ad5d4019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R32a7b5ffb9e546d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R23a774dffdee45c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R345af8af361c42cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R210201cc28d34b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Rf1bcfa65341f4375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R350139e745064551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R77bf6428b42545e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="Ra544721900914e8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Rd5d0f29e89814227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R0e5911cb94014465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="Rd5b26befd725469d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Rdb808f140fa8456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R90f7f3caabf84f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R6d012c193d26426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R17c84321d11d41db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Re6237a8f8aff43f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R46ae9685948640b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R28ba7f02190d439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R0b9815f0f18e491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="R364bae26c78b43ea"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Clean markdown from knowledge summaries
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R0e5911cb94014465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="Rd5b26befd725469d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Rdb808f140fa8456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R90f7f3caabf84f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R6d012c193d26426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R17c84321d11d41db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Re6237a8f8aff43f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R46ae9685948640b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R28ba7f02190d439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R0b9815f0f18e491b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="R364bae26c78b43ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R469c53021d9d4960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R7120f894b93d4c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Rbf6b47e8c12d4cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R7644f72eb5484905"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R550950e639834db7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R2d287c7b7cbf4ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Re3bf600c741440ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R1caaa541f40146c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="Rf0ab9838a4144614"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="Rde9d0b3853bf4b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="R9347603e780444a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -336,7 +336,7 @@
         <x:v>新能源上网电量逐步通过电力市场交易形成价格。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>新能源上网电量逐步通过电力市场交易形成价格。 ### 概念定位 新能源上网电价市场化的核心是让风电、光伏等新能源电量原则上进入电力市场，通过中长期、现货等交易形成上网价格。 对初学者来说，最重要的是把“市场交易价格”和“配套结算机制”分开看：市场交易价格来自买卖双方或现货市场出清，反映供需、时段、出力和系统运行状况； 市场价格与配套结算 配套结算机制则用于平稳衔接改革前后项目收益预期，</x:v>
+        <x:v>新能源上网电价市场化的核心是让风电、光伏等新能源电量原则上进入电力市场，通过中长期、现货等交易形成上网价格。 对初学者来说，最重要的是把“市场交易价格”和“配套结算机制”分开看：市场交易价格来自买卖双方或现货市场出清，反映供需、时段、出力和系统运行状况；</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
         <x:v>### 概念定位
@@ -379,7 +379,7 @@
         <x:v>市场经营主体参与交易前按规则完成注册的基础手续。</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
-        <x:v>市场经营主体参与交易前按规则完成注册的基础手续。 ### 概念定位 电力市场注册是发电企业、售电公司、电力用户、新型经营主体等进入电力市场前的基础管理环节。 它不是一张简单的“报名表”，而是把主体身份、经营资质、基本信息、信用和变更注销等事项纳入统一管理。 注册管理重点 注册完成后，主体才具备按规则参与市场的基础身份，但不等于自动获得所有交易品种资格；</x:v>
+        <x:v>电力市场注册是发电企业、售电公司、电力用户、新型经营主体等进入电力市场前的基础管理环节。 它不是一张简单的“报名表”，而是把主体身份、经营资质、基本信息、信用和变更注销等事项纳入统一管理。 注册管理重点 注册完成后，主体才具备按规则参与市场的基础身份，但不等于自动获得所有交易品种资格；</x:v>
       </x:c>
       <x:c r="D3" s="2" t="str">
         <x:v>### 概念定位
@@ -423,7 +423,7 @@
         <x:v>不是按发了多少电付钱，而是为电源可在关键时段顶得上、支撑系统安全供应而付的钱。</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
-        <x:v>不是按发了多少电付钱，而是为电源可在关键时段顶得上、支撑系统安全供应而付的钱。 ### 概念定位 容量电价关注的是“有没有可靠能力”，电量电价关注的是“实际发了多少电”。 传统单一制电价主要按上网电量结算，容易让煤电、气电、抽水蓄能、储能等承担保供和调节任务的电源只在发电时获得收入，难以体现其可用容量、顶峰能力和系统支撑价值。</x:v>
+        <x:v>容量电价关注的是“有没有可靠能力”，电量电价关注的是“实际发了多少电”。 传统单一制电价主要按上网电量结算，容易让煤电、气电、抽水蓄能、储能等承担保供和调节任务的电源只在发电时获得收入，难以体现其可用容量、顶峰能力和系统支撑价值。 2023年煤电容量电价机制先把合规在运公用煤电机组从单一制电价调整为两部制：电量电价由市场化方式形成，容量电价按回收一定比例固定成本确定。</x:v>
       </x:c>
       <x:c r="D4" s="2" t="str">
         <x:v>### 概念定位
@@ -471,7 +471,7 @@
         <x:v>在现货市场连续运行后，对机组在系统高峰时真正能稳定供电的能力给予补偿。</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>在现货市场连续运行后，对机组在系统高峰时真正能稳定供电的能力给予补偿。 ### 概念定位 可靠容量补偿机制比传统容量电价更强调“顶峰时能不能可靠顶上”。 2026年发电侧容量电价文件提出，电力现货市场连续运行后，省级价格主管部门会同相关部门适时建立可靠容量补偿机制，对机组可靠容量按统一原则补偿。 这里的可靠容量，是机组在全年系统顶峰时段能够持续稳定供电的容量，而不是装机容量的简单数字。</x:v>
+        <x:v>可靠容量补偿机制比传统容量电价更强调“顶峰时能不能可靠顶上”。 2026年发电侧容量电价文件提出，电力现货市场连续运行后，省级价格主管部门会同相关部门适时建立可靠容量补偿机制，对机组可靠容量按统一原则补偿。 这里的可靠容量，是机组在全年系统顶峰时段能够持续稳定供电的容量，而不是装机容量的简单数字。</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
         <x:v>### 概念定位
@@ -516,7 +516,7 @@
         <x:v>新能源价格结算机制里用于差价结算的基准价，不是新能源所有电量的固定上网电价。</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>新能源价格结算机制里用于差价结算的基准价，不是新能源所有电量的固定上网电价。 ### 概念定位 机制电价来自新能源可持续发展价格结算机制，是改革后平衡市场化交易和项目收益稳定的一项结算参数。 发改价格〔2025〕136号要求新能源上网电量原则上全部进入电力市场，价格通过市场交易形成； 同时对纳入机制的电量，电网企业每月按照机制电价开展差价结算。 结算逻辑 也就是说，新能源企业平时仍参与市场，</x:v>
+        <x:v>机制电价来自新能源可持续发展价格结算机制，是改革后平衡市场化交易和项目收益稳定的一项结算参数。 发改价格〔2025〕136号要求新能源上网电量原则上全部进入电力市场，价格通过市场交易形成； 同时对纳入机制的电量，电网企业每月按照机制电价开展差价结算。 结算逻辑 也就是说，新能源企业平时仍参与市场，市场交易均价由中长期或现货等市场形成；</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
         <x:v>### 概念定位
@@ -563,7 +563,7 @@
         <x:v>被纳入新能源可持续发展价格结算机制、可以按机制电价做差价结算的电量范围。</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>被纳入新能源可持续发展价格结算机制、可以按机制电价做差价结算的电量范围。 ### 概念定位 机制电量解决的是“哪些电量可以享受机制电价差价结算”的问题。 新能源项目上网电量原则上进入市场后，并不是全部电量都自动按机制电价结算； 只有纳入新能源可持续发展价格结算机制的电量，才会按机制电价与市场交易均价进行差价结算。 结算和清算口径 文件要求各地每年将纳入机制的电量分解到月度，</x:v>
+        <x:v>机制电量解决的是“哪些电量可以享受机制电价差价结算”的问题。 新能源项目上网电量原则上进入市场后，并不是全部电量都自动按机制电价结算； 只有纳入新能源可持续发展价格结算机制的电量，才会按机制电价与市场交易均价进行差价结算。 结算和清算口径 文件要求各地每年将纳入机制的电量分解到月度，如果某月实际上网电量低于当月分解电量，就按实际上网电量结算，并在年内按月滚动清算。</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
         <x:v>### 概念定位
@@ -609,7 +609,7 @@
         <x:v>把市场交易均价和政策机制价之间的差额算出来，多退少补式地进入结算。</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>把市场交易均价和政策机制价之间的差额算出来，多退少补式地进入结算。 ### 概念定位 差价结算是理解机制电价时最关键的结算动作。 按照新能源上网电价市场化改革文件，对纳入机制的电量，电网企业每月按机制电价开展差价结算，将市场交易均价与机制电价的差额纳入当地系统运行费用。 现货市场连续运行地区，市场交易均价原则上按月度发电侧实时市场同类项目加权平均价格确定；</x:v>
+        <x:v>差价结算是理解机制电价时最关键的结算动作。 按照新能源上网电价市场化改革文件，对纳入机制的电量，电网企业每月按机制电价开展差价结算，将市场交易均价与机制电价的差额纳入当地系统运行费用。 现货市场连续运行地区，市场交易均价原则上按月度发电侧实时市场同类项目加权平均价格确定；</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
         <x:v>### 概念定位
@@ -656,7 +656,7 @@
         <x:v>绿证证明可再生能源电量的绿色属性，绿电交易则把电能量和绿色环境价值一起交易，两者需要规则衔接避免重复计算。</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>绿证证明可再生能源电量的绿色属性，绿电交易则把电能量和绿色环境价值一起交易，两者需要规则衔接避免重复计算。 ### 概念定位 绿证市场与绿电交易衔接，是“十五五”阶段电力市场绿色价值体系的重要方向。 对初学者来说，可以把普通电力交易理解为买卖“电能量”，而绿电交易还要体现电来自可再生能源的环境价值； 绿证则是可再生能源绿色属性的凭证。 市场衔接要求 政策提出要高质量建设绿证市场，</x:v>
+        <x:v>绿证市场与绿电交易衔接，是“十五五”阶段电力市场绿色价值体系的重要方向。 对初学者来说，可以把普通电力交易理解为买卖“电能量”，而绿电交易还要体现电来自可再生能源的环境价值； 绿证则是可再生能源绿色属性的凭证。 市场衔接要求 政策提出要高质量建设绿证市场，拓展绿证应用场景，健全中长期绿证、绿电交易制度，并加强碳市场、绿证、绿电等市场化机制的衔接协同。</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
         <x:v>### 概念定位
@@ -702,7 +702,7 @@
         <x:v>通过价格信号鼓励用户在电力紧张或新能源消纳需要时调整用电，用户侧调节能力也能获得价值体现。</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>通过价格信号鼓励用户在电力紧张或新能源消纳需要时调整用电，用户侧调节能力也能获得价值体现。 ### 概念定位 需求响应价格机制关注的是用户侧调节能力。 传统电力系统更多依赖发电侧调节，新能源占比提高后，系统会更需要用户根据价格信号改变用电时间、降低尖峰负荷或配合新能源消纳。 “十五五”碳达峰行动方案提出，持续扩大电力系统调节资源规模，挖掘需求侧调节潜力，加快虚拟电厂发展，</x:v>
+        <x:v>需求响应价格机制关注的是用户侧调节能力。 传统电力系统更多依赖发电侧调节，新能源占比提高后，系统会更需要用户根据价格信号改变用电时间、降低尖峰负荷或配合新能源消纳。</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
         <x:v>### 概念定位
@@ -979,6 +979,20 @@
         <x:v>新增政策正文及附件 Markdown 提取能力，固化 OCRmyPDF + Tesseract 本地 OCR 方案，已为当前 14 个政策文件及 5 个附件生成 Markdown 原文，并为网页新增知识浏览入口。</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>更新</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>knowledgeSummary</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>清理所有知识摘要中的 Markdown 标题标记和详细解读残片，知识摘要统一为 200 字以内纯文本；结构化 Markdown 仅保留在详细解读和知识浏览中。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1041,7 +1055,7 @@
         <x:v>国家发展改革委 国家能源局关于建立煤电容量电价机制的通知</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>国家发展改革委 国家能源局关于建立煤电容量电价机制的通知。### 文件定位 该文件建立煤电容量电价机制，是从单一制煤电上网电价转向两部制电价的基础政策。 核心逻辑是把煤电收入拆成两部分：电量电价由市场化方式形成，主要反映发电量、市场供需和燃料成本； 容量电价按回收煤电机组一定比例固定成本确定，用来体现煤电在系统保供、顶峰和调节中的可用容量价值。 适用范围是合规在运的公用煤电机组，</x:v>
+        <x:v>该文件建立煤电容量电价机制，是从单一制煤电上网电价转向两部制电价的基础政策。 核心逻辑是把煤电收入拆成两部分：电量电价由市场化方式形成，主要反映发电量、市场供需和燃料成本； 容量电价按回收煤电机组一定比例固定成本确定，用来体现煤电在系统保供、顶峰和调节中的可用容量价值。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -1096,7 +1110,7 @@
         <x:v>国家发展改革委 国家能源局关于深化新能源上网电价市场化改革 促进新能源高质量发展的通知</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>国家发展改革委 国家能源局关于深化新能源上网电价市场化改革 促进新能源高质量发展的通知。### 文件定位 该文件是新能源上网电价市场化改革和机制电价、机制电量、差价结算等概念的直接来源。 文件要求风电、太阳能发电等新能源项目上网电量原则上全部进入电力市场，上网价格通过市场交易形成； 跨省跨区交易按跨省跨区市场规则形成价格。 它同时要求完善新能源参与现货和中长期市场的价格机制：现货市场中，</x:v>
+        <x:v>该文件是新能源上网电价市场化改革和机制电价、机制电量、差价结算等概念的直接来源。 文件要求风电、太阳能发电等新能源项目上网电量原则上全部进入电力市场，上网价格通过市场交易形成； 跨省跨区交易按跨省跨区市场规则形成价格。</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
         <x:v>### 文件定位
@@ -1149,7 +1163,7 @@
         <x:v>国家发展改革委 国家能源局关于完善发电侧容量电价机制的通知</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>国家发展改革委 国家能源局关于完善发电侧容量电价机制的通知。### 文件定位 该文件是在煤电容量电价机制基础上，进一步把容量价值覆盖到煤电、气电、抽水蓄能、新型储能等发电侧可靠资源的政策。 文件的核心目标是分类完善容量电价机制，既保障电力系统长期容量充裕和顶峰安全，又推动新能源高比例接入后的调节资源建设，并与现货、辅助服务、中长期交易等市场衔接。 煤电方面，</x:v>
+        <x:v>该文件是在煤电容量电价机制基础上，进一步把容量价值覆盖到煤电、气电、抽水蓄能、新型储能等发电侧可靠资源的政策。 文件的核心目标是分类完善容量电价机制，既保障电力系统长期容量充裕和顶峰安全，又推动新能源高比例接入后的调节资源建设，并与现货、辅助服务、中长期交易等市场衔接。</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
         <x:v>### 文件定位
@@ -1202,7 +1216,7 @@
         <x:v>国务院关于印发《“十五五”碳达峰行动方案》的通知</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>国务院关于印发《“十五五”碳达峰行动方案》的通知。### 文件定位和目标 该文件由国务院印发，文号为国发〔2026〕22号，生态环境部官网转载来源为中国政府网。 文件定位是“十五五”时期推进碳达峰的总纲性行动方案，目标是在2030年前确保如期实现碳达峰，并为2035年国家自主贡献目标和碳中和奠定基础。 它不是一份单一电力市场交易规则，</x:v>
+        <x:v>该文件由国务院印发，文号为国发〔2026〕22号，生态环境部官网转载来源为中国政府网。 文件定位是“十五五”时期推进碳达峰的总纲性行动方案，目标是在2030年前确保如期实现碳达峰，并为2035年国家自主贡献目标和碳中和奠定基础。</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
         <x:v>### 文件定位和目标
@@ -1262,7 +1276,7 @@
         <x:v>国家能源局关于印发《电力市场注册基本规则》的通知</x:v>
       </x:c>
       <x:c r="B6" s="2" t="str">
-        <x:v>国家能源局关于印发《电力市场注册基本规则》的通知。### 文件定位 该文件印发《电力市场注册基本规则》，有效期5年，是各地电力市场主体入市、变更、注销和信息维护的全国统一底座。 规则适用于中长期、现货、辅助服务等电力市场，覆盖发电企业、售电公司、电力用户和新型经营主体，其中新型经营主体包括新型储能、虚拟电厂、智能微电网等。 文件强调注册管理要坚持规范入市、公开透明、全国统一和信息共享，</x:v>
+        <x:v>该文件印发《电力市场注册基本规则》，有效期5年，是各地电力市场主体入市、变更、注销和信息维护的全国统一底座。 规则适用于中长期、现货、辅助服务等电力市场，覆盖发电企业、售电公司、电力用户和新型经营主体，其中新型经营主体包括新型储能、虚拟电厂、智能微电网等。</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
         <x:v>### 文件定位
@@ -1373,7 +1387,7 @@
         <x:v>关于印发《江苏省电力中长期市场实施细则（2026版）》的通知</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>关于印发《江苏省电力中长期市场实施细则（2026版）》的通知。### 文件定位 该通知发布《江苏省电力中长期市场实施细则（2026版）》，公开页面未见正式发文字号，故文号记录为“未见正式文号”。 附件细则共15章139条，是江苏省中长期市场的主要操作规则，适用于省内经营主体市场注册、交易、执行、结算、信息披露和监管。 细则首先明确经营主体包括发电企业、售电公司、电力用户和新型经营主体，</x:v>
+        <x:v>该通知发布《江苏省电力中长期市场实施细则（2026版）》，公开页面未见正式发文字号，故文号记录为“未见正式文号”。 附件细则共15章139条，是江苏省中长期市场的主要操作规则，适用于省内经营主体市场注册、交易、执行、结算、信息披露和监管。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -1491,7 +1505,7 @@
         <x:v>浙江能源监管办推动浙江电力现货市场转入正式运行</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>浙江能源监管办推动浙江电力现货市场转入正式运行。### 文件定位 浙江能源监管办公开信息显示，浙江电力现货市场于2025年8月7日转入正式运行，成为长三角地区首个正式运行的现货市场。 页面说明浙江已印发《浙江电力现货市场规则》（浙监能市场〔2024〕4号）及7个配套实施细则，形成“1+7”现货市场规则体系； 现货市场运行基础 本条来源为监管动态页面，未见可读取的7个细则附件全文，</x:v>
+        <x:v>浙江能源监管办公开信息显示，浙江电力现货市场于2025年8月7日转入正式运行，成为长三角地区首个正式运行的现货市场。 页面说明浙江已印发《浙江电力现货市场规则》（浙监能市场〔2024〕4号）及7个配套实施细则，形成“1+7”现货市场规则体系； 现货市场运行基础 本条来源为监管动态页面，未见可读取的7个细则附件全文，因此解读限于官方页面明确披露内容。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -1538,7 +1552,7 @@
         <x:v>浙江能源监管办完成电力市场三项实施细则修订</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>浙江能源监管办完成电力市场三项实施细则修订。### 文件定位 浙江能源监管办公开信息显示，其牵头完成《浙江电力现货电能量市场交易实施细则》《浙江电力调频辅助服务市场交易实施细则》和《浙江电力市场管理实施细则》三项细则修订。 公开页面没有附可读取细则全文，因此本条以官方页面列明的修订内容为依据。</x:v>
+        <x:v>浙江能源监管办公开信息显示，其牵头完成《浙江电力现货电能量市场交易实施细则》《浙江电力调频辅助服务市场交易实施细则》和《浙江电力市场管理实施细则》三项细则修订。 公开页面没有附可读取细则全文，因此本条以官方页面列明的修订内容为依据。</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
         <x:v>### 文件定位
@@ -1587,7 +1601,7 @@
         <x:v>浙江组织开展电力中长期市场等4项实施细则修订工作</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>浙江组织开展电力中长期市场等4项实施细则修订工作。### 文件定位 浙江能源监管办会同浙江省发展改革委、省能源局组织修订并公开发布《浙江电力中长期市场实施细则》《浙江电力零售市场实施细则》《浙江电力市场管理实施细则》《浙江电力市场结算实施细则》等4项细则。 公开页面为监管动态，未附可读取的四项细则全文，因此本条以页面披露的修订过程和重点问题为依据。 页面显示，</x:v>
+        <x:v>浙江能源监管办会同浙江省发展改革委、省能源局组织修订并公开发布《浙江电力中长期市场实施细则》《浙江电力零售市场实施细则》《浙江电力市场管理实施细则》《浙江电力市场结算实施细则》等4项细则。 公开页面为监管动态，未附可读取的四项细则全文，因此本条以页面披露的修订过程和重点问题为依据。</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
         <x:v>### 文件定位
@@ -1694,7 +1708,7 @@
         <x:v>山西电力中长期市场实施细则</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>山西电力中长期市场实施细则。### 文件定位 山西能源监管办公开政策解读显示，《山西电力中长期市场实施细则》（晋监能市场规〔2026〕1号）依据国家《电力中长期市场基本规则》（发改能源规〔2025〕1656号）和新能源上网电价市场化改革政策修订，结合山西电力现货市场运行实际，于2026年6月1日起施行，有效期5年，并废止原《山西电力中长期交易实施细则》（晋监能市场规〔2024〕2号）。</x:v>
+        <x:v>山西能源监管办公开政策解读显示，《山西电力中长期市场实施细则》（晋监能市场规〔2026〕1号）依据国家《电力中长期市场基本规则》（发改能源规〔2025〕1656号）和新能源上网电价市场化改革政策修订，结合山西电力现货市场运行实际，于2026年6月1日起施行，有效期5年，并废止原《山西电力中长期交易实施细则》（晋监能市场规〔2024〕2号）。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -1799,7 +1813,7 @@
         <x:v>关于印发《湖北省电力中长期市场实施细则》的通知</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>关于印发《湖北省电力中长期市场实施细则》的通知。### 文件定位 该通知由国家能源局华中监管局、湖北省发展改革委、湖北省能源局联合发布，文号为华中监能市场规﹝2026﹞39号，正文说明《湖北省电力中长期市场实施细则》已经广泛征求意见并经湖北电力市场管理委员会审议，要求电力交易机构加强经营主体宣贯培训、信息披露和风险防控。 附件细则共14章122条，</x:v>
+        <x:v>该通知由国家能源局华中监管局、湖北省发展改革委、湖北省能源局联合发布，文号为华中监能市场规﹝2026﹞39号，正文说明《湖北省电力中长期市场实施细则》已经广泛征求意见并经湖北电力市场管理委员会审议，要求电力交易机构加强经营主体宣贯培训、信息披露和风险防控。 附件细则共14章122条，适用于湖北电力中长期市场注册、交易、执行、结算、信息披露和监督管理。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -1916,7 +1930,7 @@
         <x:v>四川电力中长期市场实施细则</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>四川电力中长期市场实施细则。### 文件定位 四川能源监管办公开解读显示，《四川电力中长期市场实施细则》依据国务院办公厅关于完善全国统一电力市场体系的实施意见、《电力市场运行基本规则》《电力中长期市场基本规则》等文件制定，目的是深化四川中长期市场建设、适应全国统一电力市场和现货市场衔接需要。 公开页面为政策解读，未见可读取的正式细则附件，因此本条以官方解读确认内容为准。 解读显示，</x:v>
+        <x:v>四川能源监管办公开解读显示，《四川电力中长期市场实施细则》依据国务院办公厅关于完善全国统一电力市场体系的实施意见、《电力市场运行基本规则》《电力中长期市场基本规则》等文件制定，目的是深化四川中长期市场建设、适应全国统一电力市场和现货市场衔接需要。 公开页面为政策解读，未见可读取的正式细则附件，因此本条以官方解读确认内容为准。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -2025,7 +2039,7 @@
         <x:v>关于印发《山东电力市场规则(试行)》(2026年4月修订版)的通知</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>关于印发《山东电力市场规则(试行)》(2026年4月修订版)的通知。### 文件定位 《山东电力市场规则（试行）》（2026年4月修订版）由山东能源监管办、山东省发展改革委、山东省能源局联合印发，文号为鲁监能市场规〔2026〕27号。 通知正文要求市场运营机构严格遵循全国统一电力市场基础规则体系，规范信息披露、交易组织、交易执行、交易结算和调度运行，加快技术支持系统改造；</x:v>
+        <x:v>《山东电力市场规则（试行）》（2026年4月修订版）由山东能源监管办、山东省发展改革委、山东省能源局联合印发，文号为鲁监能市场规〔2026〕27号。 通知正文要求市场运营机构严格遵循全国统一电力市场基础规则体系，规范信息披露、交易组织、交易执行、交易结算和调度运行，加快技术支持系统改造；</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位
@@ -2142,7 +2156,7 @@
         <x:v>关于印发《甘肃省电力中长期交易实施细则》的通知</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>关于印发《甘肃省电力中长期交易实施细则》的通知。### 文件定位 该通知由国家能源局甘肃监管办公室、甘肃省发展改革委、甘肃省工信厅、甘肃省能源局联合印发，文号为甘监能市场〔2025〕212号，正文要求国网甘肃省电力公司、甘肃电力交易中心、甘肃省电力市场管理委员会以及各发电企业、售电公司、电力用户和新型经营主体遵照执行。 附件《甘肃省电力中长期交易实施细则》是本条政策的核心内容，</x:v>
+        <x:v>该通知由国家能源局甘肃监管办公室、甘肃省发展改革委、甘肃省工信厅、甘肃省能源局联合印发，文号为甘监能市场〔2025〕212号，正文要求国网甘肃省电力公司、甘肃电力交易中心、甘肃省电力市场管理委员会以及各发电企业、售电公司、电力用户和新型经营主体遵照执行。</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>### 文件定位

</xml_diff>

<commit_message>
Add logo icon to knowledge base header
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R469c53021d9d4960"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R7120f894b93d4c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Rbf6b47e8c12d4cdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="R7644f72eb5484905"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R550950e639834db7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R2d287c7b7cbf4ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Re3bf600c741440ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R1caaa541f40146c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="Rf0ab9838a4144614"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="Rde9d0b3853bf4b0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="R9347603e780444a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R3c4300245802480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R429f0e8d2f244f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R965bcedf8bad48f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="Rdcd80ff082874f12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R37f08f1621ee401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R7a3eee2299cc46cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Re296f15a2d20426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="Rdfa3c505495a492c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="Rb98d3651416b47fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R89ddc2b8a85e446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Rceaa5db91bb044b4"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add NDRC auxiliary services market rule
</commit_message>
<xml_diff>
--- a/docs/downloads/电力市场知识库-2026-07-15.xlsx
+++ b/docs/downloads/电力市场知识库-2026-07-15.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R3c4300245802480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R429f0e8d2f244f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="R965bcedf8bad48f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="Rdcd80ff082874f12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R37f08f1621ee401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R7a3eee2299cc46cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="Re296f15a2d20426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="Rdfa3c505495a492c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="Rb98d3651416b47fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R89ddc2b8a85e446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Rceaa5db91bb044b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基础概念" sheetId="1" r:id="R0ad7c5d153404314"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家政策" sheetId="2" r:id="R6c8982f84a3b4ffd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江苏" sheetId="3" r:id="Rc7ca1f6899ee438c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="浙江" sheetId="4" r:id="Ra9bca08bcbaf484e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山西" sheetId="5" r:id="R533c8be4b96f43af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="湖北" sheetId="6" r:id="R51536524788c4224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四川" sheetId="7" r:id="R0bf0980caf74442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="山东" sheetId="8" r:id="R8667d32d20554250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="甘肃" sheetId="9" r:id="R361d7ac02bdc4386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安徽" sheetId="10" r:id="R93656ec5cb56496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="11" r:id="Rea63db7b8a6a4fdd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -739,6 +739,64 @@
         <x:v>2026-07-14</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="str">
+        <x:v>电力辅助服务市场</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>不是买卖普通电量，而是用市场方式购买调峰、调频、备用、爬坡等系统稳定服务。</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>电力辅助服务市场用于购买调峰、调频、备用、爬坡等系统调节服务，帮助电网安全稳定运行，并让火电、水电、储能、虚拟电厂等可调节资源按规则获得收益或承担费用。</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>### 概念定位
+- **电力辅助服务市场**解决的不是“谁发多少电、谁买多少电”，而是电力系统运行中更隐蔽但很关键的问题：频率要稳、备用要够、峰谷要能调、新能源波动要有人快速跟上。
+- 发改能源规〔2025〕411号把辅助服务定义为：为维持电力系统安全稳定运行、保证电能质量，除正常电能生产、输送、使用之外，由可调节资源提供的调峰、调频、备用、爬坡等服务。
+### 和电能量市场的区别
+- 电能量市场主要交易“电量”和“电价”；辅助服务市场交易的是系统调节能力和实际调节效果。
+- 比如一台机组或储能系统不一定在某个时段发很多电，但它如果能按指令快速增减出力、预留备用、参与调频，就对系统安全有价值，辅助服务市场就是让这种价值被计量、出清、调用和结算。
+### 谁可以参与
+- 传统可调节电源如火电、水电通常是重要提供方；新型储能、虚拟电厂、智能微电网、车网互动运营企业等新型经营主体，也被国家规则明确纳入经营主体范围。
+- 参与主体需要具备“可观、可测、可调、可控”能力，并满足市场注册、计量通信、调度指令接收、技术支持系统接入和地方实施细则等要求。
+### 常见品种怎么理解
+- 调峰：帮助系统削峰填谷，跟随负荷峰谷和新能源出力变化调整发用电功率。
+- 调频：快速细调出力或负荷，减少频率偏差，主要包括AGC/APC等二次调频。
+- 备用：提前预留调节能力，在系统需要时按规定时间响应。
+- 爬坡：应对新能源波动或净负荷快速变化，要求资源具备较快升降出力能力。
+### 费用和考核
+- 具备市场条件的辅助服务品种通过市场交易形成价格，不同品种按调峰出力、调频里程、性能系数、中标容量、中标时间、出清价格等要素计算费用。
+- 费用传导遵循“谁受益、谁承担”。现货市场连续运行地区，符合规定的调频、备用等费用可由用户用电量和未参与电能量市场交易的上网电量共同分担；未连续运行地区原则上不向用户侧疏导辅助服务费用。
+- 经营主体如果没有按交易结果或调度指令提供有效服务，需要承担违约责任，所以辅助服务收益与真实调节能力、响应质量和履约表现直接相关。
+### 为什么重要
+- 随着新能源占比提高，风光出力波动和系统净负荷变化更明显，电力系统需要更多灵活调节资源。
+- 辅助服务市场把这种调节能力变成可交易、可结算、可考核的市场品种，是全国统一电力市场体系中与中长期、现货并列的重要组成部分。</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="str">
+        <x:v>调峰服务；调频服务；备用服务；爬坡服务；电力现货市场；虚拟电厂</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="str">
+        <x:v>国家</x:v>
+      </x:c>
+      <x:c r="G11" s="2" t="str">
+        <x:v>国家发展改革委 国家能源局关于印发《电力辅助服务市场基本规则》的通知</x:v>
+      </x:c>
+      <x:c r="H11" s="2" t="str">
+        <x:v>发改能源规〔2025〕411号</x:v>
+      </x:c>
+      <x:c r="I11" s="2" t="str">
+        <x:v>https://www.ndrc.gov.cn/xxgk/zcfb/ghxwj/202504/t20250429_1397483.html</x:v>
+      </x:c>
+      <x:c r="J11" s="2" t="str">
+        <x:v>source-files/2025-04-03-国家发展改革委 国家能源局关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号).pdf</x:v>
+      </x:c>
+      <x:c r="K11" s="2" t="str">
+        <x:v>电力辅助服务市场基本规则.pdf：source-files/attachments/2025-04-03-国家发展改革委 国家能源局关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号)/电力辅助服务市场基本规则.pdf</x:v>
+      </x:c>
+      <x:c r="L11" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -827,44 +885,44 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>2026-07-14</x:v>
+        <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>待核验</x:v>
+        <x:v>更新</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>安徽</x:v>
+        <x:v>doc-ndrc-2025-411</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
-        <x:v>未能核得安徽省电力中长期或现货市场正式有效实施细则的可访问官方链接；旧征求意见稿附件链接返回404，未作为有效政策入库。</x:v>
+        <x:v>归档发改能源规〔2025〕411号PDF正文至本地 source-files，并登记官方PDF附件用于网页“查看文件”和“附件归档”；后续同步生成Markdown原文、Excel和网页数据。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-07-14</x:v>
+        <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>新增</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
-        <x:v>doc-ndrc-2023-1501</x:v>
+        <x:v>concept-ancillary-service-market</x:v>
       </x:c>
       <x:c r="D3" s="2" t="str">
-        <x:v>补充煤电容量电价机制国家政策来源，用于支撑容量电价、容量电费等基础概念解读。</x:v>
+        <x:v>新增“电力辅助服务市场”基础概念，解释调峰、调频、备用、爬坡等辅助服务与电能量市场的区别、参与主体、费用传导和履约考核。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>2026-07-14</x:v>
+        <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
         <x:v>新增</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
-        <x:v>doc-ndrc-2026-114</x:v>
+        <x:v>doc-ndrc-2025-411</x:v>
       </x:c>
       <x:c r="D4" s="2" t="str">
-        <x:v>补充发电侧容量电价机制最新国家政策来源，用于支撑容量电价和可靠容量补偿机制解读。</x:v>
+        <x:v>新增《电力辅助服务市场基本规则》国家政策，依据国家发展改革委官网通知、附件PDF正文和官方答记者问，补充市场成员、品种、设立流程、交易组织、费用传导、结算披露、风险防控和监管要求。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -872,13 +930,13 @@
         <x:v>2026-07-14</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>新增</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>concept-capacity-electricity-price</x:v>
+        <x:v>安徽</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
-        <x:v>新增容量电价、可靠容量补偿机制、机制电价、机制电量、差价结算等基础概念，并补充详细解读。</x:v>
+        <x:v>未能核得安徽省电力中长期或现货市场正式有效实施细则的可访问官方链接；旧征求意见稿附件链接返回404，未作为有效政策入库。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -886,13 +944,13 @@
         <x:v>2026-07-14</x:v>
       </x:c>
       <x:c r="B6" s="2" t="str">
-        <x:v>更新</x:v>
+        <x:v>新增</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>provincialRules</x:v>
+        <x:v>doc-ndrc-2023-1501</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
-        <x:v>按官方来源补充江苏、浙江、山西、湖北、四川、山东、甘肃7省政策文件和省份规则摘要；安徽正式有效文件链接本轮未核得，暂不入有效规则。</x:v>
+        <x:v>补充煤电容量电价机制国家政策来源，用于支撑容量电价、容量电费等基础概念解读。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -900,13 +958,13 @@
         <x:v>2026-07-14</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
-        <x:v>更新</x:v>
+        <x:v>新增</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>policyDocuments</x:v>
+        <x:v>doc-ndrc-2026-114</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
-        <x:v>按已归档的政策网页PDF和官方附件内容，对当前已入库政策文件的详细解读逐份扩写，并同步扩写省份页可见的政策/规则总结。</x:v>
+        <x:v>补充发电侧容量电价机制最新国家政策来源，用于支撑容量电价和可靠容量补偿机制解读。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -917,29 +975,29 @@
         <x:v>新增</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>doc-state-council-2026-22</x:v>
+        <x:v>concept-capacity-electricity-price</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>根据生态环境部官网转载的国务院《“十五五”碳达峰行动方案》新增国家政策，并补充绿证市场与绿电交易衔接、需求响应价格机制等基础概念。</x:v>
+        <x:v>新增容量电价、可靠容量补偿机制、机制电价、机制电量、差价结算等基础概念，并补充详细解读。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-07-14</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
         <x:v>更新</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>concepts</x:v>
+        <x:v>provincialRules</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>按网页快速阅读要求，为已入库基础概念补充 200 字以内知识摘要，完整详细解读继续保留用于详情弹窗和 Excel 全量导出。</x:v>
+        <x:v>按官方来源补充江苏、浙江、山西、湖北、四川、山东、甘肃7省政策文件和省份规则摘要；安徽正式有效文件链接本轮未核得，暂不入有效规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-07-14</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
         <x:v>更新</x:v>
@@ -948,21 +1006,21 @@
         <x:v>policyDocuments</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
-        <x:v>按网页快速阅读要求，为已入库国家及省级政策文件补充 200 字以内知识摘要，表格展示摘要，详情保留完整详细解读。</x:v>
+        <x:v>按已归档的政策网页PDF和官方附件内容，对当前已入库政策文件的详细解读逐份扩写，并同步扩写省份页可见的政策/规则总结。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>2026-07-15</x:v>
+        <x:v>2026-07-14</x:v>
       </x:c>
       <x:c r="B11" s="2" t="str">
-        <x:v>更新</x:v>
+        <x:v>新增</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>web-preview-export-updateEvents</x:v>
+        <x:v>doc-state-council-2026-22</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
-        <x:v>优化网页头部、搜索和页签布局，删除当前页描述区域，增加导出 Excel 按钮，并固化所有知识新增、更新必须写入更新记录的维护规则。</x:v>
+        <x:v>根据生态环境部官网转载的国务院《“十五五”碳达峰行动方案》新增国家政策，并补充绿证市场与绿电交易衔接、需求响应价格机制等基础概念。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -973,10 +1031,10 @@
         <x:v>更新</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>policyDocuments</x:v>
+        <x:v>concepts</x:v>
       </x:c>
       <x:c r="D12" s="2" t="str">
-        <x:v>新增政策正文及附件 Markdown 提取能力，固化 OCRmyPDF + Tesseract 本地 OCR 方案，已为当前 14 个政策文件及 5 个附件生成 Markdown 原文，并为网页新增知识浏览入口。</x:v>
+        <x:v>按网页快速阅读要求，为已入库基础概念补充 200 字以内知识摘要，完整详细解读继续保留用于详情弹窗和 Excel 全量导出。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -987,9 +1045,51 @@
         <x:v>更新</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
+        <x:v>policyDocuments</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>按网页快速阅读要求，为已入库国家及省级政策文件补充 200 字以内知识摘要，表格展示摘要，详情保留完整详细解读。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>更新</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>web-preview-export-updateEvents</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="str">
+        <x:v>优化网页头部、搜索和页签布局，删除当前页描述区域，增加导出 Excel 按钮，并固化所有知识新增、更新必须写入更新记录的维护规则。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>更新</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>policyDocuments</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>新增政策正文及附件 Markdown 提取能力，固化 OCRmyPDF + Tesseract 本地 OCR 方案，已为当前 14 个政策文件及 5 个附件生成 Markdown 原文，并为网页新增知识浏览入口。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>更新</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
         <x:v>knowledgeSummary</x:v>
       </x:c>
-      <x:c r="D13" s="2" t="str">
+      <x:c r="D16" s="2" t="str">
         <x:v>清理所有知识摘要中的 Markdown 标题标记和详细解读残片，知识摘要统一为 200 字以内纯文本；结构化 Markdown 仅保留在详细解读和知识浏览中。</x:v>
       </x:c>
     </x:row>
@@ -1325,6 +1425,90 @@
         <x:v>2026-07-14</x:v>
       </x:c>
     </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="str">
+        <x:v>国家发展改革委 国家能源局关于印发《电力辅助服务市场基本规则》的通知</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>该文件统一规范省级及以上电力辅助服务市场，明确调峰、调频、备用、爬坡等品种，规定市场成员、设立流程、交易组织、费用传导、结算披露和监管要求。</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>### 文件定位与直接要求
+- 这是国家层面对**电力辅助服务市场**的基础性规则，正文《电力辅助服务市场基本规则》共12章67条，覆盖市场设立、注册、运行、结算、信息披露、风险防控和监管等全过程。
+- 通知正文要求国家能源局派出机构会同省级价格、能源主管部门，依据本规则和发改价格〔2024〕196号等文件，及时组织市场运营机构制修订本地区辅助服务市场实施细则，维护统一、公平的竞争制度。
+- 对已经连续运行电力现货市场的地区，文件特别要求完善现货市场规则、适当放宽市场限价，引导现货市场实现调峰功能；调峰、顶峰、调峰容量等具有类似功能的市场不再运行，避免同一系统调节价值被重复补偿。
+- 派出机构还需会同省级价格主管部门等单位，对辅助服务市场运行、资金使用、执行效果开展年度评估，重大问题及时报告国家发展改革委、国家能源局。
+### 市场是什么、为谁服务
+- 规则把电力辅助服务定义为：为维持电力系统安全稳定运行、保证电能质量，除正常电能生产、输送、使用之外，由可调节资源提供的**调峰、调频、备用、爬坡**等服务。
+- 对初学者可以理解为：电能量市场主要解决“发多少电、用多少电、什么价格成交”，辅助服务市场解决“系统怎么稳、频率怎么稳、尖峰低谷怎么调、突发波动谁来兜底”。
+- 文件的总原则是安全经济、统一开放、公平公正、竞争有序，并按照“谁提供、谁获利，谁受益、谁承担”优化价格形成和费用传导，鼓励更多可调节资源主动参与系统调节。
+### 市场成员与准入注册
+- 市场成员包括经营主体、电网企业和市场运营机构。经营主体范围不仅包括发电企业、售电企业、电力用户，也明确纳入**新型经营主体**，例如储能企业、**虚拟电厂**、智能微电网、车网互动运营企业等。
+- 能提供辅助服务的主体应满足电力市场要求，具备可观、可测、可调、可控能力，主要包括火电、水电、新型经营主体等可调节资源；获得容量电费的经营主体原则上也应参与辅助服务市场申报。
+- 经营主体原则上应具有法人资格或取得法人授权，依法取得电力业务许可证但符合豁免政策的除外，并具备独立财务核算、良好信用，以及接收和执行市场出清结果或调度指令的技术能力。
+- 经营主体必须先在电力交易机构完成市场注册，才能参与辅助服务交易；注册信息变化要办理变更，因退役、破产、政策调整、系统约束等原因退出时，要结清费用并处理未履约合同。
+### 市场如何设立和开新品种
+- 电力调度机构根据系统安全稳定运行需要、电能量市场建设情况等提出辅助服务市场建设需求，形成需求分析报告，说明本地区系统运行特点、建设必要性、影响因素和工作建议。
+- 国家能源局派出机构会同省级价格、能源主管部门组织论证需求合理性，并制定交易品种、交易机制、价格机制、限价标准、费用传导方式等实施方案；方案需报国家能源局，并经国家发展改革委同意后实施。
+- 在实施细则层面，派出机构会同省级主管部门组织市场运营机构起草规则，结合系统安全需要、服务成本、历史数据、模拟测试结果、激励效果和电价影响等确定参数，广泛征求意见并经市场管理委员会审议后发布。
+- 新设辅助服务品种不能直接“上线即结算”，需要依次开展模拟试运行、结算试运行和正式运行；首次结算试运行和正式运行开始时间间隔不少于1年，以便验证技术系统、出清结果、调度执行和费用影响。
+### 主要交易品种
+| 品种 | 规则中的核心含义 | 适合小白的理解 |
+| --- | --- | --- |
+| 调峰服务 | 跟踪负荷峰谷变化和新能源出力变化，按调度指令或出清结果调整发用电功率，包括设备启停。 | 系统低谷时少发或多用，高峰时多发或少用，帮助削峰填谷。 |
+| 调频服务 | 通过调速系统、AGC、APC等减少系统频率偏差或联络线控制偏差，主要是二次调频。 | 当系统频率轻微偏离时，快速细调出力或负荷，让电网频率稳住。 |
+| 备用服务 | 为系统安全预留调节能力，并在需要时于规定时间内调整有功出力。 | 平时先留一部分能力不全用，突发缺口时能顶上。 |
+| 爬坡服务 | 应对新能源波动等引起的净负荷短时大幅变化，由具备较强调节速率的主体按指令调整出力。 | 当净负荷突然上升或下降时，资源能快速“爬上去”或“降下来”。 |
+### 交易组织、执行和考核
+- 电力调度机构负责提出各类辅助服务需求，经营主体按公告和规则提交容量、价格、成本等交易申报；调度机构根据申报和市场规则出清，并组织调用、计费和执行记录。
+- 辅助服务市场供给不足、暂停或中止交易期间，调度机构可以为保障系统安全对应急调节资源进行调用，但事后应及时披露相关情况。
+- 经营主体如果因自身原因未按交易结果提供有效辅助服务，需要依照市场规则承担违约责任；这意味着辅助服务收益不是无条件获得，必须与实际响应能力、响应质量和履约表现绑定。
+### 费用形成与传导
+- 具备市场条件的辅助服务品种，通过市场交易形成价格；尚不具备市场条件的品种，价格机制另行规定。
+- 不同品种计费要素不同：调峰服务可按出清价格、中标调峰出力、实际调峰出力或启停次数计算；调频服务按调频里程、性能系数、出清价格等计算；备用和爬坡服务按中标容量、中标时间、出清价格等计算；提供辅助服务过程中产生的电能量费用按电能量市场规则结算。
+- 费用传导遵循“谁受益、谁承担”。现货市场未连续运行地区，原则上不向用户侧疏导辅助服务费用；现货市场连续运行地区，符合规定的调频、备用等费用原则上由用户用电量和未参与电能量市场交易的上网电量共同分担，具体比例由省级价格主管部门确定。
+- 独立储能、虚拟电厂等“发用一体”主体，在结算时段内分别按上网电量和下网电量参与发电侧、用户侧辅助服务费用分摊或分享；跨省跨区交易双方也应根据辅助服务提供和受益情况公平承担或获得费用。
+### 与现货、中长期和容量机制的衔接
+- 文件要求统筹电能量市场和辅助服务市场，在注册、交易时序、出清、费用疏导等方面衔接，避免市场割裂。
+- 调频、备用、爬坡等有功辅助服务市场可以与现货市场独立出清，具备条件时推动与现货市场联合出清；经营主体提供辅助服务产生的电能量费用仍按电能量市场规则结算。
+- 对现货连续运行地区，具有类似调峰功能的单独市场要退出或转为电能量市场功能；区域调峰、存在电能量交换的区域备用等交易，也应及时转为电能量交易。
+- 对获得容量电费的主体，规则原则上要求其参与辅助服务市场申报，体现容量补偿、可靠供给和系统调节责任之间的衔接。
+### 计量结算、披露和监管
+- 计量和采集周期应满足辅助服务最小交易周期和精度要求，数据缺失时可按拟合规则补充；结算原则上采用“日清月结”，按日清分、按月出具结算依据，辅助服务费用在电费结算单中单独列示，不得与其他费用叠加打捆。
+- 市场运营机构应披露需求计算、调用原则、需求总量、申报出清、结算等信息；经营主体对披露信息有异议的，可在规定期限内提出，交易机构和调度机构应核实处理。
+- 风险防控覆盖供需风险、市场力操纵、价格异常、技术支持系统故障、网络安全等，市场运营机构要监测预警并报告，风险处置方案需明确等级、措施和责任。
+- 国家能源局及其派出机构负责监管，市场运营机构和电网企业要按要求报送价格、费用、收入、分摊和市场运行情况；争议可通过市场运营机构、市场管理委员会调解、监管协调、仲裁或司法途径处理。
+### 对各类主体的影响
+- 发电企业尤其是火电、水电等可调节资源，需要把辅助服务作为电能量之外的重要收益与考核来源，关注报价、出清、调用、性能评价和违约责任。
+- 储能、虚拟电厂、智能微电网、车网互动运营企业等新型主体获得了国家规则层面的参与身份，但仍要满足地方细则规定的计量、通信、调控、注册和技术接入要求。
+- 电力用户和售电公司不仅可能通过聚合、虚拟电厂等方式参与提供辅助服务，在现货连续运行地区也可能按受益原则分担部分辅助服务费用，因此需要关注当地费用传导细则。
+- 省级主管部门、派出机构、调度机构和交易机构需要把本规则转化为地方实施方案、实施细则、技术系统、信息披露和年度评估机制。</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="str">
+        <x:v>发改能源规〔2025〕411号</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="str">
+        <x:v>国家发展改革委、国家能源局</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="str">
+        <x:v>2025-04-29</x:v>
+      </x:c>
+      <x:c r="G7" s="2" t="str">
+        <x:v>https://www.ndrc.gov.cn/xxgk/zcfb/ghxwj/202504/t20250429_1397483.html</x:v>
+      </x:c>
+      <x:c r="H7" s="2" t="str">
+        <x:v>source-files/2025-04-03-国家发展改革委 国家能源局关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号).pdf</x:v>
+      </x:c>
+      <x:c r="I7" s="2" t="str">
+        <x:v>电力辅助服务市场基本规则.pdf：source-files/attachments/2025-04-03-国家发展改革委 国家能源局关于印发《电力辅助服务市场基本规则》的通知(发改能源规〔2025〕411号)/电力辅助服务市场基本规则.pdf</x:v>
+      </x:c>
+      <x:c r="J7" s="2" t="str">
+        <x:v>有效</x:v>
+      </x:c>
+      <x:c r="K7" s="2" t="str">
+        <x:v>2026-07-15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>